<commit_message>
Atualiza KPIs do roadmap SEO e AEO
</commit_message>
<xml_diff>
--- a/analise/analise-seo-infinitepay.xlsx
+++ b/analise/analise-seo-infinitepay.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesll\Downloads\Teste Cloudwalk\analise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B8718A-C8BC-436C-A2C8-B09B6D8DA119}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E7E698-8AE1-460F-B048-265CE438D14E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arquitetura de páginas" sheetId="11" r:id="rId1"/>
@@ -4367,9 +4367,6 @@
     <t>Aproveitar os conteúdos existentes para apoiar o lançamento.</t>
   </si>
   <si>
-    <t>Presença da marca, páginas citadas e concorrentes.</t>
-  </si>
-  <si>
     <t>Analisar no Search Console as buscas que levam à calculadora.</t>
   </si>
   <si>
@@ -4385,9 +4382,6 @@
     <t>Usar os dados reais para orientar os próximos ajustes.</t>
   </si>
   <si>
-    <t>Evolução das citações e concorrentes mais presentes.</t>
-  </si>
-  <si>
     <t>Melhorar conteúdo e apresentação no Google nas buscas com potencial de ganho.</t>
   </si>
   <si>
@@ -4403,9 +4397,6 @@
     <t>Concentrar esforços no que os dados indicarem como oportunidade.</t>
   </si>
   <si>
-    <t>Evolução da presença e das páginas citadas desde o início.</t>
-  </si>
-  <si>
     <t>https://www.infinitepay.io/materiais/calculadora-ponto-de-equilibrio</t>
   </si>
   <si>
@@ -4413,6 +4404,15 @@
   </si>
   <si>
     <t>Página / tema*</t>
+  </si>
+  <si>
+    <t>Indexação · impressões · posição · cliques · CTR</t>
+  </si>
+  <si>
+    <t>Queries · impressões · posição · cliques · CTR</t>
+  </si>
+  <si>
+    <t>Queries · impressões · posição · cliques · CTR · referring domains</t>
   </si>
 </sst>
 </file>
@@ -4577,7 +4577,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -4609,26 +4609,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4726,16 +4713,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5445,7 +5426,14 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Base1" displayName="Base1" ref="A1:AH389" totalsRowShown="0">
-  <autoFilter ref="A1:AH389" xr:uid="{DDA5E582-3654-4FFC-8F29-F80B4F9FF6CC}"/>
+  <autoFilter ref="A1:AH389" xr:uid="{DDA5E582-3654-4FFC-8F29-F80B4F9FF6CC}">
+    <filterColumn colId="32">
+      <filters>
+        <filter val="Oportunidade"/>
+        <filter val="Vencedor"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="34">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="domain"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="keyword"/>
@@ -5512,13 +5500,7 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Base2" displayName="Base2" ref="A1:R410" totalsRowShown="0">
-  <autoFilter ref="A1:R410" xr:uid="{33CE7940-831D-4522-944D-53D92C51959C}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="False"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:R410" xr:uid="{33CE7940-831D-4522-944D-53D92C51959C}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="domain"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="keyword"/>
@@ -5774,13 +5756,13 @@
         <v>1390</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>1444</v>
+        <v>1441</v>
       </c>
       <c r="C1" s="26" t="s">
         <v>1391</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>1443</v>
+        <v>1440</v>
       </c>
       <c r="E1" s="26" t="s">
         <v>1392</v>
@@ -5799,7 +5781,7 @@
       <c r="B2" s="28" t="s">
         <v>1395</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="39" t="s">
         <v>1396</v>
       </c>
       <c r="D2" s="28" t="s">
@@ -5822,7 +5804,7 @@
       <c r="B3" s="25" t="s">
         <v>1401</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="38" t="s">
         <v>1402</v>
       </c>
       <c r="D3" s="25" t="s">
@@ -5845,7 +5827,7 @@
       <c r="B4" s="28" t="s">
         <v>1406</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="39" t="s">
         <v>1407</v>
       </c>
       <c r="D4" s="28" t="s">
@@ -5868,8 +5850,8 @@
       <c r="B5" s="25" t="s">
         <v>1344</v>
       </c>
-      <c r="C5" s="40" t="s">
-        <v>1442</v>
+      <c r="C5" s="38" t="s">
+        <v>1439</v>
       </c>
       <c r="D5" s="25" t="s">
         <v>1413</v>
@@ -5891,7 +5873,7 @@
       <c r="B6" s="28" t="s">
         <v>1417</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="39" t="s">
         <v>1314</v>
       </c>
       <c r="D6" s="28" t="s">
@@ -5965,7 +5947,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="79.2">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="37" t="s">
         <v>1384</v>
       </c>
       <c r="B2" s="33" t="s">
@@ -5983,8 +5965,8 @@
       <c r="F2" s="34" t="s">
         <v>1428</v>
       </c>
-      <c r="G2" s="35" t="s">
-        <v>1429</v>
+      <c r="G2" s="17" t="s">
+        <v>1442</v>
       </c>
       <c r="H2" s="17" t="s">
         <v>1385</v>
@@ -5994,49 +5976,49 @@
       <c r="A3" s="29" t="s">
         <v>1386</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="35" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C3" s="36" t="s">
         <v>1430</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="D3" s="36" t="s">
         <v>1431</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="E3" s="36" t="s">
         <v>1432</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="F3" s="36" t="s">
         <v>1433</v>
       </c>
-      <c r="F3" s="37" t="s">
-        <v>1434</v>
-      </c>
-      <c r="G3" s="38" t="s">
-        <v>1435</v>
+      <c r="G3" s="16" t="s">
+        <v>1443</v>
       </c>
       <c r="H3" s="16" t="s">
         <v>1387</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="52.8">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="37" t="s">
         <v>1388</v>
       </c>
       <c r="B4" s="33" t="s">
+        <v>1434</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>1435</v>
+      </c>
+      <c r="D4" s="34" t="s">
         <v>1436</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="E4" s="34" t="s">
         <v>1437</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="F4" s="34" t="s">
         <v>1438</v>
       </c>
-      <c r="E4" s="34" t="s">
-        <v>1439</v>
-      </c>
-      <c r="F4" s="34" t="s">
-        <v>1440</v>
-      </c>
-      <c r="G4" s="35" t="s">
-        <v>1441</v>
+      <c r="G4" s="15" t="s">
+        <v>1444</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>1389</v>
@@ -6328,7 +6310,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="15" customHeight="1">
+    <row r="2" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -6432,7 +6414,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="15" customHeight="1">
+    <row r="3" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>37</v>
       </c>
@@ -6536,7 +6518,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="4" spans="1:34" ht="15" customHeight="1">
+    <row r="4" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
@@ -6640,7 +6622,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="5" spans="1:34" ht="15" customHeight="1">
+    <row r="5" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>60</v>
       </c>
@@ -6742,7 +6724,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="6" spans="1:34" ht="15" customHeight="1">
+    <row r="6" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>140</v>
       </c>
@@ -6846,7 +6828,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="7" spans="1:34" ht="15" customHeight="1">
+    <row r="7" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>101</v>
       </c>
@@ -6948,7 +6930,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="8" spans="1:34" ht="15" customHeight="1">
+    <row r="8" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>54</v>
       </c>
@@ -7050,7 +7032,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="9" spans="1:34" ht="15" customHeight="1">
+    <row r="9" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>101</v>
       </c>
@@ -7154,7 +7136,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="10" spans="1:34" ht="15" customHeight="1">
+    <row r="10" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
@@ -7258,7 +7240,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="11" spans="1:34" ht="15" customHeight="1">
+    <row r="11" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>25</v>
       </c>
@@ -7362,7 +7344,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="12" spans="1:34" ht="15" customHeight="1">
+    <row r="12" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>65</v>
       </c>
@@ -7456,7 +7438,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="13" spans="1:34" ht="15" customHeight="1">
+    <row r="13" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>60</v>
       </c>
@@ -7558,7 +7540,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="14" spans="1:34" ht="15" customHeight="1">
+    <row r="14" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>37</v>
       </c>
@@ -7660,7 +7642,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="15" spans="1:34" ht="15" customHeight="1">
+    <row r="15" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>54</v>
       </c>
@@ -7762,7 +7744,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="16" spans="1:34" ht="15" customHeight="1">
+    <row r="16" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>82</v>
       </c>
@@ -7866,7 +7848,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="17" spans="1:34" ht="15" customHeight="1">
+    <row r="17" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
@@ -7970,7 +7952,7 @@
         <v>1345</v>
       </c>
     </row>
-    <row r="18" spans="1:34" ht="15" customHeight="1">
+    <row r="18" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
@@ -8072,7 +8054,7 @@
         <v>1345</v>
       </c>
     </row>
-    <row r="19" spans="1:34" ht="15" customHeight="1">
+    <row r="19" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>173</v>
       </c>
@@ -8176,7 +8158,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="20" spans="1:34" ht="15" customHeight="1">
+    <row r="20" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>82</v>
       </c>
@@ -8278,7 +8260,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="21" spans="1:34" ht="15" customHeight="1">
+    <row r="21" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>82</v>
       </c>
@@ -8382,7 +8364,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="22" spans="1:34" ht="15" customHeight="1">
+    <row r="22" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>51</v>
       </c>
@@ -8484,7 +8466,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="23" spans="1:34" ht="15" customHeight="1">
+    <row r="23" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>82</v>
       </c>
@@ -8586,7 +8568,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="24" spans="1:34" ht="15" customHeight="1">
+    <row r="24" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>88</v>
       </c>
@@ -8688,7 +8670,7 @@
         <v>1345</v>
       </c>
     </row>
-    <row r="25" spans="1:34" ht="15" customHeight="1">
+    <row r="25" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>42</v>
       </c>
@@ -8790,7 +8772,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="26" spans="1:34" ht="15" customHeight="1">
+    <row r="26" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>140</v>
       </c>
@@ -8892,7 +8874,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="27" spans="1:34" ht="15" customHeight="1">
+    <row r="27" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A27" s="1" t="s">
         <v>54</v>
       </c>
@@ -8996,7 +8978,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="28" spans="1:34" ht="15" customHeight="1">
+    <row r="28" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A28" s="1" t="s">
         <v>82</v>
       </c>
@@ -9100,7 +9082,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="29" spans="1:34" ht="15" customHeight="1">
+    <row r="29" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A29" s="1" t="s">
         <v>51</v>
       </c>
@@ -9204,7 +9186,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="30" spans="1:34" ht="15" customHeight="1">
+    <row r="30" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>54</v>
       </c>
@@ -9308,7 +9290,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="31" spans="1:34" ht="15" customHeight="1">
+    <row r="31" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>82</v>
       </c>
@@ -9412,7 +9394,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="32" spans="1:34" ht="15" customHeight="1">
+    <row r="32" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A32" s="1" t="s">
         <v>54</v>
       </c>
@@ -9514,7 +9496,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="33" spans="1:34" ht="15" customHeight="1">
+    <row r="33" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A33" s="1" t="s">
         <v>54</v>
       </c>
@@ -9616,7 +9598,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="34" spans="1:34" ht="15" customHeight="1">
+    <row r="34" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A34" s="1" t="s">
         <v>51</v>
       </c>
@@ -9718,7 +9700,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="35" spans="1:34" ht="15" customHeight="1">
+    <row r="35" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A35" s="1" t="s">
         <v>51</v>
       </c>
@@ -9822,7 +9804,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="36" spans="1:34" ht="15" customHeight="1">
+    <row r="36" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A36" s="1" t="s">
         <v>82</v>
       </c>
@@ -9926,7 +9908,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="37" spans="1:34" ht="15" customHeight="1">
+    <row r="37" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A37" s="1" t="s">
         <v>60</v>
       </c>
@@ -10028,7 +10010,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="38" spans="1:34" ht="15" customHeight="1">
+    <row r="38" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
@@ -10235,7 +10217,7 @@
         <v>Maior potencial orgânico, mas menor conexão com a jornada de gestão financeira do lojista.</v>
       </c>
     </row>
-    <row r="40" spans="1:34" ht="24" customHeight="1">
+    <row r="40" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A40" s="1" t="s">
         <v>25</v>
       </c>
@@ -10337,7 +10319,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="41" spans="1:34" ht="15" customHeight="1">
+    <row r="41" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A41" s="1" t="s">
         <v>37</v>
       </c>
@@ -10439,7 +10421,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="42" spans="1:34" ht="15" customHeight="1">
+    <row r="42" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A42" s="1" t="s">
         <v>25</v>
       </c>
@@ -10646,7 +10628,7 @@
         <v>Boa demanda, mas intenção mais informacional/regulatória do que de uso de ferramenta.</v>
       </c>
     </row>
-    <row r="44" spans="1:34" ht="15" customHeight="1">
+    <row r="44" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A44" s="1" t="s">
         <v>39</v>
       </c>
@@ -10750,7 +10732,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="45" spans="1:34" ht="15" customHeight="1">
+    <row r="45" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A45" s="1" t="s">
         <v>82</v>
       </c>
@@ -10852,7 +10834,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="46" spans="1:34" ht="15" customHeight="1">
+    <row r="46" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A46" s="1" t="s">
         <v>65</v>
       </c>
@@ -10946,7 +10928,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="47" spans="1:34" ht="15" customHeight="1">
+    <row r="47" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A47" s="1" t="s">
         <v>42</v>
       </c>
@@ -11050,7 +11032,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="48" spans="1:34" ht="15" customHeight="1">
+    <row r="48" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A48" s="1" t="s">
         <v>42</v>
       </c>
@@ -11152,7 +11134,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="49" spans="1:34" ht="15" customHeight="1">
+    <row r="49" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A49" s="1" t="s">
         <v>120</v>
       </c>
@@ -11256,7 +11238,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="50" spans="1:34" ht="15" customHeight="1">
+    <row r="50" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A50" s="1" t="s">
         <v>88</v>
       </c>
@@ -11461,7 +11443,7 @@
         <v>Excelente potencial orgânico, mas menor aderência ao negócio e ao ecossistema da InfinitePay.</v>
       </c>
     </row>
-    <row r="52" spans="1:34" ht="15" customHeight="1">
+    <row r="52" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A52" s="1" t="s">
         <v>39</v>
       </c>
@@ -11563,7 +11545,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="53" spans="1:34" ht="15" customHeight="1">
+    <row r="53" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A53" s="1" t="s">
         <v>60</v>
       </c>
@@ -11667,7 +11649,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="54" spans="1:34" ht="15" customHeight="1">
+    <row r="54" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A54" s="1" t="s">
         <v>25</v>
       </c>
@@ -11769,7 +11751,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="55" spans="1:34" ht="15" customHeight="1">
+    <row r="55" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A55" s="1" t="s">
         <v>25</v>
       </c>
@@ -11873,7 +11855,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="56" spans="1:34" ht="15" customHeight="1">
+    <row r="56" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A56" s="1" t="s">
         <v>65</v>
       </c>
@@ -11969,7 +11951,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="57" spans="1:34" ht="15" customHeight="1">
+    <row r="57" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A57" s="1" t="s">
         <v>51</v>
       </c>
@@ -12071,7 +12053,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="58" spans="1:34" ht="15" customHeight="1">
+    <row r="58" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A58" s="1" t="s">
         <v>65</v>
       </c>
@@ -12167,7 +12149,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="59" spans="1:34" ht="15" customHeight="1">
+    <row r="59" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A59" s="1" t="s">
         <v>25</v>
       </c>
@@ -12477,7 +12459,7 @@
         <v>Forte oportunidade, mas muito próxima da Calculadora de Preço de Venda que a InfinitePay já possui.</v>
       </c>
     </row>
-    <row r="62" spans="1:34" ht="24" customHeight="1">
+    <row r="62" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A62" s="1" t="s">
         <v>120</v>
       </c>
@@ -12579,7 +12561,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="63" spans="1:34" ht="15" customHeight="1">
+    <row r="63" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A63" s="1" t="s">
         <v>39</v>
       </c>
@@ -12683,7 +12665,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="64" spans="1:34" ht="15" customHeight="1">
+    <row r="64" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A64" s="1" t="s">
         <v>60</v>
       </c>
@@ -12787,7 +12769,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="65" spans="1:34" ht="15" customHeight="1">
+    <row r="65" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A65" s="1" t="s">
         <v>39</v>
       </c>
@@ -12891,7 +12873,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="66" spans="1:34" ht="15" customHeight="1">
+    <row r="66" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A66" s="1" t="s">
         <v>42</v>
       </c>
@@ -12993,7 +12975,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="67" spans="1:34" ht="15" customHeight="1">
+    <row r="67" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A67" s="1" t="s">
         <v>25</v>
       </c>
@@ -13097,7 +13079,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="68" spans="1:34" ht="15" customHeight="1">
+    <row r="68" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A68" s="1" t="s">
         <v>60</v>
       </c>
@@ -13201,7 +13183,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="69" spans="1:34" ht="15" customHeight="1">
+    <row r="69" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A69" s="1" t="s">
         <v>140</v>
       </c>
@@ -13303,7 +13285,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="70" spans="1:34" ht="15" customHeight="1">
+    <row r="70" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A70" s="1" t="s">
         <v>54</v>
       </c>
@@ -13405,7 +13387,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="71" spans="1:34" ht="15" customHeight="1">
+    <row r="71" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A71" s="1" t="s">
         <v>173</v>
       </c>
@@ -13507,7 +13489,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="72" spans="1:34" ht="15" customHeight="1">
+    <row r="72" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A72" s="1" t="s">
         <v>140</v>
       </c>
@@ -13609,7 +13591,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="73" spans="1:34" ht="15" customHeight="1">
+    <row r="73" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A73" s="1" t="s">
         <v>54</v>
       </c>
@@ -13713,7 +13695,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="74" spans="1:34" ht="15" customHeight="1">
+    <row r="74" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A74" s="1" t="s">
         <v>54</v>
       </c>
@@ -13815,7 +13797,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="75" spans="1:34" ht="15" customHeight="1">
+    <row r="75" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A75" s="1" t="s">
         <v>54</v>
       </c>
@@ -13917,7 +13899,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="76" spans="1:34" ht="15" customHeight="1">
+    <row r="76" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A76" s="1" t="s">
         <v>42</v>
       </c>
@@ -14021,7 +14003,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="77" spans="1:34" ht="15" customHeight="1">
+    <row r="77" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A77" s="1" t="s">
         <v>37</v>
       </c>
@@ -14123,7 +14105,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="78" spans="1:34" ht="15" customHeight="1">
+    <row r="78" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A78" s="1" t="s">
         <v>120</v>
       </c>
@@ -14225,7 +14207,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="79" spans="1:34" ht="15" customHeight="1">
+    <row r="79" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A79" s="1" t="s">
         <v>82</v>
       </c>
@@ -14327,7 +14309,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="80" spans="1:34" ht="15" customHeight="1">
+    <row r="80" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A80" s="1" t="s">
         <v>65</v>
       </c>
@@ -14423,7 +14405,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="81" spans="1:34" ht="15" customHeight="1">
+    <row r="81" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A81" s="1" t="s">
         <v>120</v>
       </c>
@@ -14525,7 +14507,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="82" spans="1:34" ht="15" customHeight="1">
+    <row r="82" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A82" s="1" t="s">
         <v>54</v>
       </c>
@@ -14627,7 +14609,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="83" spans="1:34" ht="15" customHeight="1">
+    <row r="83" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A83" s="1" t="s">
         <v>173</v>
       </c>
@@ -14729,7 +14711,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="84" spans="1:34" ht="15" customHeight="1">
+    <row r="84" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -14833,7 +14815,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="85" spans="1:34" ht="15" customHeight="1">
+    <row r="85" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A85" s="1" t="s">
         <v>54</v>
       </c>
@@ -14935,7 +14917,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="86" spans="1:34" ht="15" customHeight="1">
+    <row r="86" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A86" s="1" t="s">
         <v>82</v>
       </c>
@@ -15037,7 +15019,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="87" spans="1:34" ht="15" customHeight="1">
+    <row r="87" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A87" s="1" t="s">
         <v>51</v>
       </c>
@@ -15141,7 +15123,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="88" spans="1:34" ht="15" customHeight="1">
+    <row r="88" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A88" s="1" t="s">
         <v>51</v>
       </c>
@@ -15243,7 +15225,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="89" spans="1:34" ht="15" customHeight="1">
+    <row r="89" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A89" s="1" t="s">
         <v>101</v>
       </c>
@@ -15345,7 +15327,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="90" spans="1:34" ht="15" customHeight="1">
+    <row r="90" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A90" s="1" t="s">
         <v>173</v>
       </c>
@@ -15447,7 +15429,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="91" spans="1:34" ht="15" customHeight="1">
+    <row r="91" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A91" s="1" t="s">
         <v>54</v>
       </c>
@@ -15549,7 +15531,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="92" spans="1:34" ht="15" customHeight="1">
+    <row r="92" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A92" s="1" t="s">
         <v>51</v>
       </c>
@@ -15651,7 +15633,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="93" spans="1:34" ht="15" customHeight="1">
+    <row r="93" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A93" s="1" t="s">
         <v>42</v>
       </c>
@@ -15753,7 +15735,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="94" spans="1:34" ht="15" customHeight="1">
+    <row r="94" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A94" s="1" t="s">
         <v>39</v>
       </c>
@@ -15855,7 +15837,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="95" spans="1:34" ht="15" customHeight="1">
+    <row r="95" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A95" s="1" t="s">
         <v>42</v>
       </c>
@@ -15959,7 +15941,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="96" spans="1:34" ht="15" customHeight="1">
+    <row r="96" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A96" s="1" t="s">
         <v>65</v>
       </c>
@@ -16055,7 +16037,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="97" spans="1:34" ht="15" customHeight="1">
+    <row r="97" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A97" s="1" t="s">
         <v>37</v>
       </c>
@@ -16157,7 +16139,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="98" spans="1:34" ht="15" customHeight="1">
+    <row r="98" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A98" s="1" t="s">
         <v>88</v>
       </c>
@@ -16261,7 +16243,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="99" spans="1:34" ht="15" customHeight="1">
+    <row r="99" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A99" s="1" t="s">
         <v>25</v>
       </c>
@@ -16363,7 +16345,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="100" spans="1:34" ht="15" customHeight="1">
+    <row r="100" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A100" s="1" t="s">
         <v>173</v>
       </c>
@@ -16465,7 +16447,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="101" spans="1:34" ht="24" customHeight="1">
+    <row r="101" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A101" s="1" t="s">
         <v>54</v>
       </c>
@@ -16569,7 +16551,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="102" spans="1:34" ht="15" customHeight="1">
+    <row r="102" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A102" s="1" t="s">
         <v>65</v>
       </c>
@@ -16665,7 +16647,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="103" spans="1:34" ht="15" customHeight="1">
+    <row r="103" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A103" s="1" t="s">
         <v>25</v>
       </c>
@@ -16769,7 +16751,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="104" spans="1:34" ht="15" customHeight="1">
+    <row r="104" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A104" s="1" t="s">
         <v>60</v>
       </c>
@@ -16871,7 +16853,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="105" spans="1:34" ht="15" customHeight="1">
+    <row r="105" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A105" s="1" t="s">
         <v>65</v>
       </c>
@@ -16965,7 +16947,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="106" spans="1:34" ht="15" customHeight="1">
+    <row r="106" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A106" s="1" t="s">
         <v>88</v>
       </c>
@@ -17069,7 +17051,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="107" spans="1:34" ht="15" customHeight="1">
+    <row r="107" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A107" s="1" t="s">
         <v>37</v>
       </c>
@@ -17173,7 +17155,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="108" spans="1:34" ht="15" customHeight="1">
+    <row r="108" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A108" s="1" t="s">
         <v>88</v>
       </c>
@@ -17275,7 +17257,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="109" spans="1:34" ht="15" customHeight="1">
+    <row r="109" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A109" s="1" t="s">
         <v>82</v>
       </c>
@@ -17377,7 +17359,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="110" spans="1:34" ht="15" customHeight="1">
+    <row r="110" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A110" s="1" t="s">
         <v>120</v>
       </c>
@@ -17481,7 +17463,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="111" spans="1:34" ht="15" customHeight="1">
+    <row r="111" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A111" s="1" t="s">
         <v>37</v>
       </c>
@@ -17583,7 +17565,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="112" spans="1:34" ht="15" customHeight="1">
+    <row r="112" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A112" s="1" t="s">
         <v>39</v>
       </c>
@@ -17687,7 +17669,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="113" spans="1:34" ht="15" customHeight="1">
+    <row r="113" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A113" s="1" t="s">
         <v>140</v>
       </c>
@@ -17789,7 +17771,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="114" spans="1:34" ht="15" customHeight="1">
+    <row r="114" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A114" s="1" t="s">
         <v>65</v>
       </c>
@@ -18091,7 +18073,7 @@
         <v>Bom fit com lojistas, mas a intenção observada é predominantemente informacional.</v>
       </c>
     </row>
-    <row r="117" spans="1:34" ht="15" customHeight="1">
+    <row r="117" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A117" s="1" t="s">
         <v>91</v>
       </c>
@@ -18195,7 +18177,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="118" spans="1:34" ht="15" customHeight="1">
+    <row r="118" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A118" s="1" t="s">
         <v>54</v>
       </c>
@@ -18400,7 +18382,7 @@
         <v>Tema aderente ao negócio, mas a busca indica intenção principalmente explicativa.</v>
       </c>
     </row>
-    <row r="120" spans="1:34" ht="15" customHeight="1">
+    <row r="120" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A120" s="1" t="s">
         <v>37</v>
       </c>
@@ -18502,7 +18484,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="121" spans="1:34" ht="15" customHeight="1">
+    <row r="121" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A121" s="1" t="s">
         <v>42</v>
       </c>
@@ -18606,7 +18588,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="122" spans="1:34" ht="15" customHeight="1">
+    <row r="122" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A122" s="1" t="s">
         <v>39</v>
       </c>
@@ -18708,7 +18690,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="123" spans="1:34" ht="15" customHeight="1">
+    <row r="123" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A123" s="1" t="s">
         <v>65</v>
       </c>
@@ -18804,7 +18786,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="124" spans="1:34" ht="15" customHeight="1">
+    <row r="124" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A124" s="1" t="s">
         <v>120</v>
       </c>
@@ -18908,7 +18890,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="125" spans="1:34" ht="15" customHeight="1">
+    <row r="125" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A125" s="1" t="s">
         <v>42</v>
       </c>
@@ -19012,7 +18994,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="126" spans="1:34" ht="15" customHeight="1">
+    <row r="126" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A126" s="1" t="s">
         <v>88</v>
       </c>
@@ -19114,7 +19096,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="127" spans="1:34" ht="15" customHeight="1">
+    <row r="127" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A127" s="1" t="s">
         <v>91</v>
       </c>
@@ -19216,7 +19198,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="128" spans="1:34" ht="15" customHeight="1">
+    <row r="128" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A128" s="1" t="s">
         <v>42</v>
       </c>
@@ -19320,7 +19302,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="129" spans="1:34" ht="15" customHeight="1">
+    <row r="129" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A129" s="1" t="s">
         <v>39</v>
       </c>
@@ -19422,7 +19404,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="130" spans="1:34" ht="15" customHeight="1">
+    <row r="130" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A130" s="1" t="s">
         <v>25</v>
       </c>
@@ -19526,7 +19508,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="131" spans="1:34" ht="15" customHeight="1">
+    <row r="131" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A131" s="1" t="s">
         <v>82</v>
       </c>
@@ -19630,7 +19612,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="132" spans="1:34" ht="15" customHeight="1">
+    <row r="132" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A132" s="1" t="s">
         <v>91</v>
       </c>
@@ -19732,7 +19714,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="133" spans="1:34" ht="15" customHeight="1">
+    <row r="133" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A133" s="1" t="s">
         <v>88</v>
       </c>
@@ -19834,7 +19816,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="134" spans="1:34" ht="15" customHeight="1">
+    <row r="134" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A134" s="1" t="s">
         <v>82</v>
       </c>
@@ -19938,7 +19920,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="135" spans="1:34" ht="15" customHeight="1">
+    <row r="135" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A135" s="1" t="s">
         <v>91</v>
       </c>
@@ -20042,7 +20024,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="136" spans="1:34" ht="15" customHeight="1">
+    <row r="136" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A136" s="1" t="s">
         <v>88</v>
       </c>
@@ -20144,7 +20126,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="137" spans="1:34" ht="15" customHeight="1">
+    <row r="137" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A137" s="1" t="s">
         <v>140</v>
       </c>
@@ -20246,7 +20228,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="138" spans="1:34" ht="15" customHeight="1">
+    <row r="138" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A138" s="1" t="s">
         <v>140</v>
       </c>
@@ -20348,7 +20330,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="139" spans="1:34" ht="15" customHeight="1">
+    <row r="139" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A139" s="1" t="s">
         <v>82</v>
       </c>
@@ -20450,7 +20432,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="140" spans="1:34" ht="15" customHeight="1">
+    <row r="140" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A140" s="1" t="s">
         <v>65</v>
       </c>
@@ -20544,7 +20526,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="141" spans="1:34" ht="15" customHeight="1">
+    <row r="141" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A141" s="1" t="s">
         <v>39</v>
       </c>
@@ -20646,7 +20628,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="142" spans="1:34" ht="15" customHeight="1">
+    <row r="142" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A142" s="1" t="s">
         <v>37</v>
       </c>
@@ -20748,7 +20730,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="143" spans="1:34" ht="15" customHeight="1">
+    <row r="143" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A143" s="1" t="s">
         <v>101</v>
       </c>
@@ -20850,7 +20832,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="144" spans="1:34" ht="15" customHeight="1">
+    <row r="144" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A144" s="1" t="s">
         <v>173</v>
       </c>
@@ -21055,7 +21037,7 @@
         <v>Tema financeiro relevante, mas a intenção está mais ligada a produto/informação do que a uma ferramenta.</v>
       </c>
     </row>
-    <row r="146" spans="1:34" ht="15" customHeight="1">
+    <row r="146" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A146" s="1" t="s">
         <v>88</v>
       </c>
@@ -21157,7 +21139,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="147" spans="1:34" ht="15" customHeight="1">
+    <row r="147" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A147" s="1" t="s">
         <v>120</v>
       </c>
@@ -21261,7 +21243,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="148" spans="1:34" ht="15" customHeight="1">
+    <row r="148" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A148" s="1" t="s">
         <v>65</v>
       </c>
@@ -21357,7 +21339,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="149" spans="1:34" ht="15" customHeight="1">
+    <row r="149" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A149" s="1" t="s">
         <v>42</v>
       </c>
@@ -21459,7 +21441,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="150" spans="1:34" ht="15" customHeight="1">
+    <row r="150" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A150" s="1" t="s">
         <v>88</v>
       </c>
@@ -21561,7 +21543,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="151" spans="1:34" ht="15" customHeight="1">
+    <row r="151" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A151" s="1" t="s">
         <v>60</v>
       </c>
@@ -21663,7 +21645,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="152" spans="1:34" ht="15" customHeight="1">
+    <row r="152" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A152" s="1" t="s">
         <v>65</v>
       </c>
@@ -21757,7 +21739,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="153" spans="1:34" ht="15" customHeight="1">
+    <row r="153" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A153" s="1" t="s">
         <v>60</v>
       </c>
@@ -21861,7 +21843,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="154" spans="1:34" ht="15" customHeight="1">
+    <row r="154" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A154" s="1" t="s">
         <v>120</v>
       </c>
@@ -21963,7 +21945,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="155" spans="1:34" ht="15" customHeight="1">
+    <row r="155" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A155" s="1" t="s">
         <v>51</v>
       </c>
@@ -22067,7 +22049,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="156" spans="1:34" ht="15" customHeight="1">
+    <row r="156" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A156" s="1" t="s">
         <v>65</v>
       </c>
@@ -22163,7 +22145,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="157" spans="1:34" ht="15" customHeight="1">
+    <row r="157" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A157" s="1" t="s">
         <v>120</v>
       </c>
@@ -22267,7 +22249,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="158" spans="1:34" ht="15" customHeight="1">
+    <row r="158" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A158" s="1" t="s">
         <v>39</v>
       </c>
@@ -22371,7 +22353,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="159" spans="1:34" ht="15" customHeight="1">
+    <row r="159" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A159" s="1" t="s">
         <v>60</v>
       </c>
@@ -22473,7 +22455,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="160" spans="1:34" ht="15" customHeight="1">
+    <row r="160" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A160" s="1" t="s">
         <v>37</v>
       </c>
@@ -22575,7 +22557,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="161" spans="1:34" ht="15" customHeight="1">
+    <row r="161" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A161" s="1" t="s">
         <v>42</v>
       </c>
@@ -22677,7 +22659,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="162" spans="1:34" ht="15" customHeight="1">
+    <row r="162" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A162" s="1" t="s">
         <v>60</v>
       </c>
@@ -22779,7 +22761,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="163" spans="1:34" ht="15" customHeight="1">
+    <row r="163" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A163" s="1" t="s">
         <v>37</v>
       </c>
@@ -22883,7 +22865,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="164" spans="1:34" ht="15" customHeight="1">
+    <row r="164" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A164" s="1" t="s">
         <v>120</v>
       </c>
@@ -22985,7 +22967,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="165" spans="1:34" ht="15" customHeight="1">
+    <row r="165" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A165" s="1" t="s">
         <v>37</v>
       </c>
@@ -23087,7 +23069,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="166" spans="1:34" ht="15" customHeight="1">
+    <row r="166" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A166" s="1" t="s">
         <v>54</v>
       </c>
@@ -23189,7 +23171,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="167" spans="1:34" ht="15" customHeight="1">
+    <row r="167" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A167" s="1" t="s">
         <v>39</v>
       </c>
@@ -23293,7 +23275,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="168" spans="1:34" ht="15" customHeight="1">
+    <row r="168" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A168" s="1" t="s">
         <v>39</v>
       </c>
@@ -23397,7 +23379,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="169" spans="1:34" ht="15" customHeight="1">
+    <row r="169" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A169" s="1" t="s">
         <v>65</v>
       </c>
@@ -23493,7 +23475,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="170" spans="1:34" ht="15" customHeight="1">
+    <row r="170" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A170" s="1" t="s">
         <v>140</v>
       </c>
@@ -23597,7 +23579,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="171" spans="1:34" ht="15" customHeight="1">
+    <row r="171" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A171" s="1" t="s">
         <v>120</v>
       </c>
@@ -23699,7 +23681,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="172" spans="1:34" ht="15" customHeight="1">
+    <row r="172" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A172" s="1" t="s">
         <v>42</v>
       </c>
@@ -23803,7 +23785,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="173" spans="1:34" ht="15" customHeight="1">
+    <row r="173" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A173" s="1" t="s">
         <v>54</v>
       </c>
@@ -24008,7 +23990,7 @@
         <v>ESCOLHIDA — melhor equilíbrio entre demanda, fit com o lojista, formato de ferramenta e ecossistema existente.</v>
       </c>
     </row>
-    <row r="175" spans="1:34" ht="15" customHeight="1">
+    <row r="175" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A175" s="1" t="s">
         <v>65</v>
       </c>
@@ -24102,7 +24084,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="176" spans="1:34" ht="15" customHeight="1">
+    <row r="176" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A176" s="1" t="s">
         <v>91</v>
       </c>
@@ -24204,7 +24186,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="177" spans="1:34" ht="15" customHeight="1">
+    <row r="177" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A177" s="1" t="s">
         <v>91</v>
       </c>
@@ -24413,7 +24395,7 @@
         <v>ESCOLHIDA — melhor equilíbrio entre demanda, fit com o lojista, formato de ferramenta e ecossistema existente.</v>
       </c>
     </row>
-    <row r="179" spans="1:34" ht="15" customHeight="1">
+    <row r="179" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A179" s="1" t="s">
         <v>91</v>
       </c>
@@ -24517,7 +24499,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="180" spans="1:34" ht="15" customHeight="1">
+    <row r="180" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A180" s="1" t="s">
         <v>140</v>
       </c>
@@ -24621,7 +24603,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="181" spans="1:34" ht="15" customHeight="1">
+    <row r="181" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A181" s="1" t="s">
         <v>91</v>
       </c>
@@ -24725,7 +24707,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="182" spans="1:34" ht="15" customHeight="1">
+    <row r="182" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A182" s="1" t="s">
         <v>37</v>
       </c>
@@ -24829,7 +24811,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="183" spans="1:34" ht="15" customHeight="1">
+    <row r="183" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A183" s="1" t="s">
         <v>25</v>
       </c>
@@ -24931,7 +24913,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="184" spans="1:34" ht="15" customHeight="1">
+    <row r="184" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A184" s="1" t="s">
         <v>88</v>
       </c>
@@ -25035,7 +25017,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="185" spans="1:34" ht="15" customHeight="1">
+    <row r="185" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A185" s="1" t="s">
         <v>65</v>
       </c>
@@ -25129,7 +25111,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="186" spans="1:34" ht="15" customHeight="1">
+    <row r="186" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A186" s="1" t="s">
         <v>37</v>
       </c>
@@ -25231,7 +25213,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="187" spans="1:34" ht="24" customHeight="1">
+    <row r="187" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A187" s="1" t="s">
         <v>88</v>
       </c>
@@ -25333,7 +25315,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="188" spans="1:34" ht="15" customHeight="1">
+    <row r="188" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A188" s="1" t="s">
         <v>88</v>
       </c>
@@ -25435,7 +25417,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="189" spans="1:34" ht="15" customHeight="1">
+    <row r="189" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A189" s="1" t="s">
         <v>65</v>
       </c>
@@ -25529,7 +25511,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="190" spans="1:34" ht="15" customHeight="1">
+    <row r="190" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A190" s="1" t="s">
         <v>65</v>
       </c>
@@ -25625,7 +25607,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="191" spans="1:34" ht="15" customHeight="1">
+    <row r="191" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A191" s="1" t="s">
         <v>42</v>
       </c>
@@ -25727,7 +25709,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="192" spans="1:34" ht="15" customHeight="1">
+    <row r="192" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A192" s="1" t="s">
         <v>88</v>
       </c>
@@ -25829,7 +25811,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="193" spans="1:34" ht="15" customHeight="1">
+    <row r="193" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A193" s="1" t="s">
         <v>51</v>
       </c>
@@ -25931,7 +25913,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="194" spans="1:34" ht="15" customHeight="1">
+    <row r="194" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A194" s="1" t="s">
         <v>101</v>
       </c>
@@ -26033,7 +26015,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="195" spans="1:34" ht="15" customHeight="1">
+    <row r="195" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A195" s="1" t="s">
         <v>173</v>
       </c>
@@ -26135,7 +26117,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="196" spans="1:34" ht="15" customHeight="1">
+    <row r="196" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A196" s="1" t="s">
         <v>65</v>
       </c>
@@ -26229,7 +26211,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="197" spans="1:34" ht="15" customHeight="1">
+    <row r="197" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A197" s="1" t="s">
         <v>65</v>
       </c>
@@ -26323,7 +26305,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="198" spans="1:34" ht="15" customHeight="1">
+    <row r="198" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A198" s="1" t="s">
         <v>120</v>
       </c>
@@ -26427,7 +26409,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="199" spans="1:34" ht="15" customHeight="1">
+    <row r="199" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A199" s="1" t="s">
         <v>88</v>
       </c>
@@ -26529,7 +26511,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="200" spans="1:34" ht="15" customHeight="1">
+    <row r="200" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A200" s="1" t="s">
         <v>65</v>
       </c>
@@ -26623,7 +26605,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="201" spans="1:34" ht="24" customHeight="1">
+    <row r="201" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A201" s="1" t="s">
         <v>140</v>
       </c>
@@ -26727,7 +26709,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="202" spans="1:34" ht="15" customHeight="1">
+    <row r="202" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A202" s="1" t="s">
         <v>120</v>
       </c>
@@ -26829,7 +26811,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="203" spans="1:34" ht="15" customHeight="1">
+    <row r="203" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A203" s="1" t="s">
         <v>65</v>
       </c>
@@ -26925,7 +26907,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="204" spans="1:34" ht="15" customHeight="1">
+    <row r="204" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A204" s="1" t="s">
         <v>39</v>
       </c>
@@ -27029,7 +27011,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="205" spans="1:34" ht="15" customHeight="1">
+    <row r="205" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A205" s="1" t="s">
         <v>60</v>
       </c>
@@ -27131,7 +27113,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="206" spans="1:34" ht="24" customHeight="1">
+    <row r="206" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A206" s="1" t="s">
         <v>37</v>
       </c>
@@ -27235,7 +27217,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="207" spans="1:34" ht="15" customHeight="1">
+    <row r="207" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A207" s="1" t="s">
         <v>39</v>
       </c>
@@ -27337,7 +27319,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="208" spans="1:34" ht="15" customHeight="1">
+    <row r="208" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A208" s="1" t="s">
         <v>65</v>
       </c>
@@ -27431,7 +27413,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="209" spans="1:34" ht="15" customHeight="1">
+    <row r="209" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A209" s="1" t="s">
         <v>88</v>
       </c>
@@ -27533,7 +27515,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="210" spans="1:34" ht="15" customHeight="1">
+    <row r="210" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A210" s="1" t="s">
         <v>60</v>
       </c>
@@ -27738,7 +27720,7 @@
         <v>É calculável, mas funciona melhor como parte da jornada de ponto de equilíbrio do que como ferramenta isolada.</v>
       </c>
     </row>
-    <row r="212" spans="1:34" ht="15" customHeight="1">
+    <row r="212" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A212" s="1" t="s">
         <v>37</v>
       </c>
@@ -27842,7 +27824,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="213" spans="1:34" ht="15" customHeight="1">
+    <row r="213" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A213" s="1" t="s">
         <v>37</v>
       </c>
@@ -28049,7 +28031,7 @@
         <v>É calculável, mas funciona melhor como parte da jornada de ponto de equilíbrio do que como ferramenta isolada.</v>
       </c>
     </row>
-    <row r="215" spans="1:34" ht="15" customHeight="1">
+    <row r="215" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A215" s="1" t="s">
         <v>120</v>
       </c>
@@ -28153,7 +28135,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="216" spans="1:34" ht="15" customHeight="1">
+    <row r="216" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A216" s="1" t="s">
         <v>39</v>
       </c>
@@ -28255,7 +28237,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="217" spans="1:34" ht="15" customHeight="1">
+    <row r="217" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A217" s="1" t="s">
         <v>42</v>
       </c>
@@ -28359,7 +28341,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="218" spans="1:34" ht="15" customHeight="1">
+    <row r="218" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A218" s="1" t="s">
         <v>91</v>
       </c>
@@ -28463,7 +28445,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="219" spans="1:34" ht="15" customHeight="1">
+    <row r="219" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A219" s="1" t="s">
         <v>60</v>
       </c>
@@ -28565,7 +28547,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="220" spans="1:34" ht="15" customHeight="1">
+    <row r="220" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A220" s="1" t="s">
         <v>88</v>
       </c>
@@ -28667,7 +28649,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="221" spans="1:34" ht="15" customHeight="1">
+    <row r="221" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A221" s="1" t="s">
         <v>140</v>
       </c>
@@ -28769,7 +28751,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="222" spans="1:34" ht="15" customHeight="1">
+    <row r="222" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A222" s="1" t="s">
         <v>60</v>
       </c>
@@ -28873,7 +28855,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="223" spans="1:34" ht="15" customHeight="1">
+    <row r="223" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A223" s="1" t="s">
         <v>37</v>
       </c>
@@ -28975,7 +28957,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="224" spans="1:34" ht="15" customHeight="1">
+    <row r="224" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A224" s="1" t="s">
         <v>37</v>
       </c>
@@ -29079,7 +29061,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="225" spans="1:34" ht="15" customHeight="1">
+    <row r="225" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A225" s="1" t="s">
         <v>65</v>
       </c>
@@ -29175,7 +29157,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="226" spans="1:34" ht="15" customHeight="1">
+    <row r="226" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A226" s="1" t="s">
         <v>39</v>
       </c>
@@ -29277,7 +29259,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="227" spans="1:34" ht="15" customHeight="1">
+    <row r="227" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A227" s="1" t="s">
         <v>54</v>
       </c>
@@ -29379,7 +29361,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="228" spans="1:34" ht="15" customHeight="1">
+    <row r="228" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A228" s="1" t="s">
         <v>54</v>
       </c>
@@ -29481,7 +29463,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="229" spans="1:34" ht="15" customHeight="1">
+    <row r="229" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A229" s="1" t="s">
         <v>51</v>
       </c>
@@ -29583,7 +29565,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="230" spans="1:34" ht="15" customHeight="1">
+    <row r="230" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A230" s="1" t="s">
         <v>82</v>
       </c>
@@ -29685,7 +29667,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="231" spans="1:34" ht="15" customHeight="1">
+    <row r="231" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A231" s="1" t="s">
         <v>91</v>
       </c>
@@ -29789,7 +29771,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="232" spans="1:34" ht="15" customHeight="1">
+    <row r="232" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A232" s="1" t="s">
         <v>101</v>
       </c>
@@ -29891,7 +29873,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="233" spans="1:34" ht="15" customHeight="1">
+    <row r="233" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A233" s="1" t="s">
         <v>54</v>
       </c>
@@ -29995,7 +29977,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="234" spans="1:34" ht="15" customHeight="1">
+    <row r="234" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A234" s="1" t="s">
         <v>173</v>
       </c>
@@ -30099,7 +30081,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="235" spans="1:34" ht="15" customHeight="1">
+    <row r="235" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A235" s="1" t="s">
         <v>54</v>
       </c>
@@ -30201,7 +30183,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="236" spans="1:34" ht="15" customHeight="1">
+    <row r="236" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A236" s="1" t="s">
         <v>65</v>
       </c>
@@ -30295,7 +30277,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="237" spans="1:34" ht="15" customHeight="1">
+    <row r="237" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A237" s="1" t="s">
         <v>101</v>
       </c>
@@ -30397,7 +30379,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="238" spans="1:34" ht="15" customHeight="1">
+    <row r="238" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A238" s="1" t="s">
         <v>54</v>
       </c>
@@ -30499,7 +30481,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="239" spans="1:34" ht="15" customHeight="1">
+    <row r="239" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A239" s="1" t="s">
         <v>173</v>
       </c>
@@ -30601,7 +30583,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="240" spans="1:34" ht="15" customHeight="1">
+    <row r="240" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A240" s="1" t="s">
         <v>101</v>
       </c>
@@ -30703,7 +30685,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="241" spans="1:34" ht="15" customHeight="1">
+    <row r="241" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A241" s="1" t="s">
         <v>101</v>
       </c>
@@ -30805,7 +30787,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="242" spans="1:34" ht="15" customHeight="1">
+    <row r="242" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A242" s="1" t="s">
         <v>54</v>
       </c>
@@ -30907,7 +30889,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="243" spans="1:34" ht="24" customHeight="1">
+    <row r="243" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A243" s="1" t="s">
         <v>101</v>
       </c>
@@ -31009,7 +30991,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="244" spans="1:34" ht="15" customHeight="1">
+    <row r="244" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A244" s="1" t="s">
         <v>173</v>
       </c>
@@ -31113,7 +31095,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="245" spans="1:34" ht="15" customHeight="1">
+    <row r="245" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A245" s="1" t="s">
         <v>54</v>
       </c>
@@ -31215,7 +31197,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="246" spans="1:34" ht="15" customHeight="1">
+    <row r="246" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A246" s="1" t="s">
         <v>54</v>
       </c>
@@ -31317,7 +31299,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="247" spans="1:34" ht="15" customHeight="1">
+    <row r="247" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A247" s="1" t="s">
         <v>51</v>
       </c>
@@ -31421,7 +31403,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="248" spans="1:34" ht="15" customHeight="1">
+    <row r="248" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A248" s="1" t="s">
         <v>37</v>
       </c>
@@ -31525,7 +31507,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="249" spans="1:34" ht="15" customHeight="1">
+    <row r="249" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A249" s="1" t="s">
         <v>91</v>
       </c>
@@ -31629,7 +31611,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="250" spans="1:34" ht="15" customHeight="1">
+    <row r="250" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A250" s="1" t="s">
         <v>51</v>
       </c>
@@ -31733,7 +31715,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="251" spans="1:34" ht="15" customHeight="1">
+    <row r="251" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A251" s="1" t="s">
         <v>120</v>
       </c>
@@ -31837,7 +31819,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="252" spans="1:34" ht="15" customHeight="1">
+    <row r="252" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A252" s="1" t="s">
         <v>88</v>
       </c>
@@ -31939,7 +31921,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="253" spans="1:34" ht="15" customHeight="1">
+    <row r="253" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A253" s="1" t="s">
         <v>60</v>
       </c>
@@ -32041,7 +32023,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="254" spans="1:34" ht="15" customHeight="1">
+    <row r="254" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A254" s="1" t="s">
         <v>42</v>
       </c>
@@ -32143,7 +32125,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="255" spans="1:34" ht="15" customHeight="1">
+    <row r="255" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A255" s="1" t="s">
         <v>37</v>
       </c>
@@ -32247,7 +32229,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="256" spans="1:34" ht="15" customHeight="1">
+    <row r="256" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A256" s="1" t="s">
         <v>88</v>
       </c>
@@ -32456,7 +32438,7 @@
         <v>Tem fit com lojistas, mas “vale a pena” indica uma necessidade mais editorial do que operacional.</v>
       </c>
     </row>
-    <row r="258" spans="1:34" ht="15" customHeight="1">
+    <row r="258" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A258" s="1" t="s">
         <v>65</v>
       </c>
@@ -32550,7 +32532,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="259" spans="1:34" ht="15" customHeight="1">
+    <row r="259" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A259" s="1" t="s">
         <v>42</v>
       </c>
@@ -32652,7 +32634,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="260" spans="1:34" ht="15" customHeight="1">
+    <row r="260" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A260" s="1" t="s">
         <v>65</v>
       </c>
@@ -32746,7 +32728,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="261" spans="1:34" ht="15" customHeight="1">
+    <row r="261" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A261" s="1" t="s">
         <v>120</v>
       </c>
@@ -32848,7 +32830,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="262" spans="1:34" ht="15" customHeight="1">
+    <row r="262" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A262" s="1" t="s">
         <v>37</v>
       </c>
@@ -32950,7 +32932,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="263" spans="1:34" ht="15" customHeight="1">
+    <row r="263" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A263" s="1" t="s">
         <v>39</v>
       </c>
@@ -33052,7 +33034,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="264" spans="1:34" ht="15" customHeight="1">
+    <row r="264" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A264" s="1" t="s">
         <v>120</v>
       </c>
@@ -33154,7 +33136,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="265" spans="1:34" ht="15" customHeight="1">
+    <row r="265" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A265" s="1" t="s">
         <v>120</v>
       </c>
@@ -33256,7 +33238,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="266" spans="1:34" ht="15" customHeight="1">
+    <row r="266" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A266" s="1" t="s">
         <v>42</v>
       </c>
@@ -33463,7 +33445,7 @@
         <v>É calculável, mas tem aplicação mais específica e intenção de ferramenta menos evidente.</v>
       </c>
     </row>
-    <row r="268" spans="1:34" ht="15" customHeight="1">
+    <row r="268" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A268" s="1" t="s">
         <v>88</v>
       </c>
@@ -33565,7 +33547,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="269" spans="1:34" ht="15" customHeight="1">
+    <row r="269" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A269" s="1" t="s">
         <v>42</v>
       </c>
@@ -33667,7 +33649,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="270" spans="1:34" ht="15" customHeight="1">
+    <row r="270" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A270" s="1" t="s">
         <v>65</v>
       </c>
@@ -33866,7 +33848,7 @@
         <v>Pode virar ferramenta, mas apresenta oportunidade orgânica e intenção menos fortes que os finalistas.</v>
       </c>
     </row>
-    <row r="272" spans="1:34" ht="15" customHeight="1">
+    <row r="272" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A272" s="1" t="s">
         <v>88</v>
       </c>
@@ -33968,7 +33950,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="273" spans="1:34" ht="15" customHeight="1">
+    <row r="273" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A273" s="1" t="s">
         <v>37</v>
       </c>
@@ -34072,7 +34054,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="274" spans="1:34" ht="24" customHeight="1">
+    <row r="274" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A274" s="1" t="s">
         <v>65</v>
       </c>
@@ -34168,7 +34150,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="275" spans="1:34" ht="15" customHeight="1">
+    <row r="275" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A275" s="1" t="s">
         <v>120</v>
       </c>
@@ -34272,7 +34254,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="276" spans="1:34" ht="15" customHeight="1">
+    <row r="276" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A276" s="1" t="s">
         <v>39</v>
       </c>
@@ -34376,7 +34358,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="277" spans="1:34" ht="15" customHeight="1">
+    <row r="277" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A277" s="1" t="s">
         <v>60</v>
       </c>
@@ -34478,7 +34460,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="278" spans="1:34" ht="15" customHeight="1">
+    <row r="278" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A278" s="1" t="s">
         <v>60</v>
       </c>
@@ -34582,7 +34564,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="279" spans="1:34" ht="15" customHeight="1">
+    <row r="279" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A279" s="1" t="s">
         <v>37</v>
       </c>
@@ -34684,7 +34666,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="280" spans="1:34" ht="15" customHeight="1">
+    <row r="280" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A280" s="1" t="s">
         <v>91</v>
       </c>
@@ -34788,7 +34770,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="281" spans="1:34" ht="15" customHeight="1">
+    <row r="281" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A281" s="1" t="s">
         <v>54</v>
       </c>
@@ -34993,7 +34975,7 @@
         <v>Ferramenta bastante clara, mas com demanda menor e aplicação mais específica.</v>
       </c>
     </row>
-    <row r="283" spans="1:34" ht="15" customHeight="1">
+    <row r="283" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A283" s="1" t="s">
         <v>120</v>
       </c>
@@ -35095,7 +35077,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="284" spans="1:34" ht="15" customHeight="1">
+    <row r="284" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A284" s="1" t="s">
         <v>37</v>
       </c>
@@ -35197,7 +35179,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="285" spans="1:34" ht="15" customHeight="1">
+    <row r="285" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A285" s="1" t="s">
         <v>88</v>
       </c>
@@ -35299,7 +35281,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="286" spans="1:34" ht="15" customHeight="1">
+    <row r="286" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A286" s="1" t="s">
         <v>39</v>
       </c>
@@ -35403,7 +35385,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="287" spans="1:34" ht="15" customHeight="1">
+    <row r="287" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A287" s="1" t="s">
         <v>65</v>
       </c>
@@ -35497,7 +35479,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="288" spans="1:34" ht="15" customHeight="1">
+    <row r="288" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A288" s="1" t="s">
         <v>140</v>
       </c>
@@ -35601,7 +35583,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="289" spans="1:34" ht="15" customHeight="1">
+    <row r="289" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A289" s="1" t="s">
         <v>91</v>
       </c>
@@ -35705,7 +35687,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="290" spans="1:34" ht="15" customHeight="1">
+    <row r="290" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A290" s="1" t="s">
         <v>120</v>
       </c>
@@ -35809,7 +35791,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="291" spans="1:34" ht="15" customHeight="1">
+    <row r="291" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A291" s="1" t="s">
         <v>54</v>
       </c>
@@ -35911,7 +35893,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="292" spans="1:34" ht="15" customHeight="1">
+    <row r="292" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A292" s="1" t="s">
         <v>51</v>
       </c>
@@ -36013,7 +35995,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="293" spans="1:34" ht="15" customHeight="1">
+    <row r="293" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A293" s="1" t="s">
         <v>82</v>
       </c>
@@ -36117,7 +36099,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="294" spans="1:34" ht="15" customHeight="1">
+    <row r="294" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A294" s="1" t="s">
         <v>51</v>
       </c>
@@ -36219,7 +36201,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="295" spans="1:34" ht="15" customHeight="1">
+    <row r="295" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A295" s="1" t="s">
         <v>60</v>
       </c>
@@ -36321,7 +36303,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="296" spans="1:34" ht="15" customHeight="1">
+    <row r="296" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A296" s="1" t="s">
         <v>82</v>
       </c>
@@ -36423,7 +36405,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="297" spans="1:34" ht="15" customHeight="1">
+    <row r="297" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A297" s="1" t="s">
         <v>54</v>
       </c>
@@ -36527,7 +36509,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="298" spans="1:34" ht="15" customHeight="1">
+    <row r="298" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A298" s="1" t="s">
         <v>82</v>
       </c>
@@ -36631,7 +36613,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="299" spans="1:34" ht="15" customHeight="1">
+    <row r="299" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A299" s="1" t="s">
         <v>51</v>
       </c>
@@ -36733,7 +36715,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="300" spans="1:34" ht="15" customHeight="1">
+    <row r="300" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A300" s="1" t="s">
         <v>140</v>
       </c>
@@ -36835,7 +36817,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="301" spans="1:34" ht="15" customHeight="1">
+    <row r="301" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A301" s="1" t="s">
         <v>65</v>
       </c>
@@ -36931,7 +36913,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="302" spans="1:34" ht="15" customHeight="1">
+    <row r="302" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A302" s="1" t="s">
         <v>51</v>
       </c>
@@ -37035,7 +37017,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="303" spans="1:34" ht="15" customHeight="1">
+    <row r="303" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A303" s="1" t="s">
         <v>54</v>
       </c>
@@ -37139,7 +37121,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="304" spans="1:34" ht="15" customHeight="1">
+    <row r="304" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A304" s="1" t="s">
         <v>54</v>
       </c>
@@ -37243,7 +37225,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="305" spans="1:34" ht="15" customHeight="1">
+    <row r="305" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A305" s="1" t="s">
         <v>54</v>
       </c>
@@ -37345,7 +37327,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="306" spans="1:34" ht="15" customHeight="1">
+    <row r="306" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A306" s="1" t="s">
         <v>39</v>
       </c>
@@ -37449,7 +37431,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="307" spans="1:34" ht="15" customHeight="1">
+    <row r="307" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A307" s="1" t="s">
         <v>140</v>
       </c>
@@ -37553,7 +37535,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="308" spans="1:34" ht="24" customHeight="1">
+    <row r="308" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A308" s="1" t="s">
         <v>60</v>
       </c>
@@ -37863,7 +37845,7 @@
         <v>Tema importante para precificação, mas a intenção é principalmente comparar e entender os conceitos.</v>
       </c>
     </row>
-    <row r="311" spans="1:34" ht="15" customHeight="1">
+    <row r="311" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A311" s="1" t="s">
         <v>65</v>
       </c>
@@ -37957,7 +37939,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="312" spans="1:34" ht="15" customHeight="1">
+    <row r="312" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A312" s="1" t="s">
         <v>39</v>
       </c>
@@ -38061,7 +38043,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="313" spans="1:34" ht="15" customHeight="1">
+    <row r="313" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A313" s="1" t="s">
         <v>60</v>
       </c>
@@ -38165,7 +38147,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="314" spans="1:34" ht="15" customHeight="1">
+    <row r="314" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A314" s="1" t="s">
         <v>42</v>
       </c>
@@ -38267,7 +38249,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="315" spans="1:34" ht="15" customHeight="1">
+    <row r="315" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A315" s="1" t="s">
         <v>42</v>
       </c>
@@ -38369,7 +38351,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="316" spans="1:34" ht="15" customHeight="1">
+    <row r="316" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A316" s="1" t="s">
         <v>65</v>
       </c>
@@ -38463,7 +38445,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="317" spans="1:34" ht="15" customHeight="1">
+    <row r="317" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A317" s="1" t="s">
         <v>37</v>
       </c>
@@ -38565,7 +38547,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="318" spans="1:34" ht="15" customHeight="1">
+    <row r="318" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A318" s="1" t="s">
         <v>42</v>
       </c>
@@ -38669,7 +38651,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="319" spans="1:34" ht="15" customHeight="1">
+    <row r="319" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A319" s="1" t="s">
         <v>120</v>
       </c>
@@ -38771,7 +38753,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="320" spans="1:34" ht="15" customHeight="1">
+    <row r="320" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A320" s="1" t="s">
         <v>173</v>
       </c>
@@ -38875,7 +38857,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="321" spans="1:34" ht="15" customHeight="1">
+    <row r="321" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A321" s="1" t="s">
         <v>37</v>
       </c>
@@ -38977,7 +38959,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="322" spans="1:34" ht="15" customHeight="1">
+    <row r="322" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A322" s="1" t="s">
         <v>88</v>
       </c>
@@ -39079,7 +39061,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="323" spans="1:34" ht="15" customHeight="1">
+    <row r="323" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A323" s="1" t="s">
         <v>88</v>
       </c>
@@ -39181,7 +39163,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="324" spans="1:34" ht="15" customHeight="1">
+    <row r="324" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A324" s="1" t="s">
         <v>140</v>
       </c>
@@ -39596,7 +39578,7 @@
         <v>É calculável e aderente à gestão, mas possui demanda menor e intenção de ferramenta menos explícita.</v>
       </c>
     </row>
-    <row r="328" spans="1:34" ht="15" customHeight="1">
+    <row r="328" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A328" s="1" t="s">
         <v>42</v>
       </c>
@@ -39803,7 +39785,7 @@
         <v>É calculável e aderente à gestão, mas possui demanda menor e intenção de ferramenta menos explícita.</v>
       </c>
     </row>
-    <row r="330" spans="1:34" ht="15" customHeight="1">
+    <row r="330" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A330" s="1" t="s">
         <v>60</v>
       </c>
@@ -39907,7 +39889,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="331" spans="1:34" ht="15" customHeight="1">
+    <row r="331" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A331" s="1" t="s">
         <v>88</v>
       </c>
@@ -40011,7 +39993,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="332" spans="1:34" ht="15" customHeight="1">
+    <row r="332" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A332" s="1" t="s">
         <v>82</v>
       </c>
@@ -40218,7 +40200,7 @@
         <v>Oportunidade específica, de menor demanda e dentro de um território de precificação já explorado.</v>
       </c>
     </row>
-    <row r="334" spans="1:34" ht="24" customHeight="1">
+    <row r="334" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A334" s="1" t="s">
         <v>82</v>
       </c>
@@ -40320,7 +40302,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="335" spans="1:34" ht="15" customHeight="1">
+    <row r="335" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A335" s="1" t="s">
         <v>25</v>
       </c>
@@ -40422,7 +40404,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="336" spans="1:34" ht="15" customHeight="1">
+    <row r="336" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A336" s="1" t="s">
         <v>82</v>
       </c>
@@ -40524,7 +40506,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="337" spans="1:34" ht="15" customHeight="1">
+    <row r="337" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A337" s="1" t="s">
         <v>120</v>
       </c>
@@ -40626,7 +40608,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="338" spans="1:34" ht="15" customHeight="1">
+    <row r="338" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A338" s="1" t="s">
         <v>39</v>
       </c>
@@ -40728,7 +40710,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="339" spans="1:34" ht="15" customHeight="1">
+    <row r="339" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A339" s="1" t="s">
         <v>88</v>
       </c>
@@ -40830,7 +40812,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="340" spans="1:34" ht="15" customHeight="1">
+    <row r="340" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A340" s="1" t="s">
         <v>39</v>
       </c>
@@ -40934,7 +40916,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="341" spans="1:34" ht="15" customHeight="1">
+    <row r="341" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A341" s="1" t="s">
         <v>25</v>
       </c>
@@ -41036,7 +41018,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="342" spans="1:34" ht="15" customHeight="1">
+    <row r="342" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A342" s="1" t="s">
         <v>140</v>
       </c>
@@ -41243,7 +41225,7 @@
         <v>Pode apoiar uma ferramenta, mas “passo a passo” indica forte componente tutorial.</v>
       </c>
     </row>
-    <row r="344" spans="1:34" ht="15" customHeight="1">
+    <row r="344" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A344" s="1" t="s">
         <v>91</v>
       </c>
@@ -41450,7 +41432,7 @@
         <v>Boa intenção para ferramenta, mas com escala orgânica muito inferior aos principais candidatos.</v>
       </c>
     </row>
-    <row r="346" spans="1:34" ht="15" customHeight="1">
+    <row r="346" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A346" s="1" t="s">
         <v>42</v>
       </c>
@@ -41552,7 +41534,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="347" spans="1:34" ht="15" customHeight="1">
+    <row r="347" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A347" s="1" t="s">
         <v>88</v>
       </c>
@@ -41654,7 +41636,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="348" spans="1:34" ht="15" customHeight="1">
+    <row r="348" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A348" s="1" t="s">
         <v>91</v>
       </c>
@@ -41964,7 +41946,7 @@
         <v>Tem aderência ao lojista, mas o modificador “2026” reforça uma intenção de conteúdo atualizado.</v>
       </c>
     </row>
-    <row r="351" spans="1:34" ht="15" customHeight="1">
+    <row r="351" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A351" s="1" t="s">
         <v>120</v>
       </c>
@@ -42068,7 +42050,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="352" spans="1:34" ht="15" customHeight="1">
+    <row r="352" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A352" s="1" t="s">
         <v>39</v>
       </c>
@@ -42170,7 +42152,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="353" spans="1:34" ht="15" customHeight="1">
+    <row r="353" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A353" s="1" t="s">
         <v>25</v>
       </c>
@@ -42274,7 +42256,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="354" spans="1:34" ht="15" customHeight="1">
+    <row r="354" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A354" s="1" t="s">
         <v>88</v>
       </c>
@@ -42378,7 +42360,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="355" spans="1:34" ht="15" customHeight="1">
+    <row r="355" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A355" s="1" t="s">
         <v>82</v>
       </c>
@@ -42482,7 +42464,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="356" spans="1:34" ht="15" customHeight="1">
+    <row r="356" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A356" s="1" t="s">
         <v>120</v>
       </c>
@@ -42586,7 +42568,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="357" spans="1:34" ht="15" customHeight="1">
+    <row r="357" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A357" s="1" t="s">
         <v>88</v>
       </c>
@@ -42793,7 +42775,7 @@
         <v>Ótima intenção de ferramenta, mas baixa demanda e forte proximidade com a calculadora de preço existente.</v>
       </c>
     </row>
-    <row r="359" spans="1:34" ht="15" customHeight="1">
+    <row r="359" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A359" s="1" t="s">
         <v>51</v>
       </c>
@@ -42895,7 +42877,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="360" spans="1:34" ht="15" customHeight="1">
+    <row r="360" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A360" s="1" t="s">
         <v>54</v>
       </c>
@@ -42997,7 +42979,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="361" spans="1:34" ht="15" customHeight="1">
+    <row r="361" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A361" s="1" t="s">
         <v>54</v>
       </c>
@@ -43101,7 +43083,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="362" spans="1:34" ht="15" customHeight="1">
+    <row r="362" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A362" s="1" t="s">
         <v>82</v>
       </c>
@@ -43203,7 +43185,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="363" spans="1:34" ht="15" customHeight="1">
+    <row r="363" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A363" s="1" t="s">
         <v>140</v>
       </c>
@@ -43307,7 +43289,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="364" spans="1:34" ht="15" customHeight="1">
+    <row r="364" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A364" s="1" t="s">
         <v>82</v>
       </c>
@@ -43411,7 +43393,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="365" spans="1:34" ht="15" customHeight="1">
+    <row r="365" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A365" s="1" t="s">
         <v>37</v>
       </c>
@@ -43513,7 +43495,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="366" spans="1:34" ht="15" customHeight="1">
+    <row r="366" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A366" s="1" t="s">
         <v>120</v>
       </c>
@@ -43617,7 +43599,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="367" spans="1:34" ht="15" customHeight="1">
+    <row r="367" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A367" s="1" t="s">
         <v>37</v>
       </c>
@@ -43721,7 +43703,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="368" spans="1:34" ht="15" customHeight="1">
+    <row r="368" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A368" s="1" t="s">
         <v>60</v>
       </c>
@@ -43823,7 +43805,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="369" spans="1:34" ht="15" customHeight="1">
+    <row r="369" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A369" s="1" t="s">
         <v>65</v>
       </c>
@@ -43917,7 +43899,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="370" spans="1:34" ht="15" customHeight="1">
+    <row r="370" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A370" s="1" t="s">
         <v>51</v>
       </c>
@@ -44019,7 +44001,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="371" spans="1:34" ht="15" customHeight="1">
+    <row r="371" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A371" s="1" t="s">
         <v>60</v>
       </c>
@@ -44121,7 +44103,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="372" spans="1:34" ht="15" customHeight="1">
+    <row r="372" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A372" s="1" t="s">
         <v>37</v>
       </c>
@@ -44225,7 +44207,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="373" spans="1:34" ht="15" customHeight="1">
+    <row r="373" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A373" s="1" t="s">
         <v>37</v>
       </c>
@@ -44434,7 +44416,7 @@
         <v>Tema relevante para empresas, mas predominantemente fiscal/informacional e mais complexo de manter como ferramenta.</v>
       </c>
     </row>
-    <row r="375" spans="1:34" ht="15" customHeight="1">
+    <row r="375" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A375" s="1" t="s">
         <v>39</v>
       </c>
@@ -44538,7 +44520,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="376" spans="1:34" ht="15" customHeight="1">
+    <row r="376" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A376" s="1" t="s">
         <v>88</v>
       </c>
@@ -44640,7 +44622,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="377" spans="1:34" ht="15" customHeight="1">
+    <row r="377" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A377" s="1" t="s">
         <v>39</v>
       </c>
@@ -44744,7 +44726,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="378" spans="1:34" ht="15" customHeight="1">
+    <row r="378" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A378" s="1" t="s">
         <v>120</v>
       </c>
@@ -44848,7 +44830,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="379" spans="1:34" ht="15" customHeight="1">
+    <row r="379" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A379" s="1" t="s">
         <v>88</v>
       </c>
@@ -44952,7 +44934,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="380" spans="1:34" ht="15" customHeight="1">
+    <row r="380" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A380" s="1" t="s">
         <v>39</v>
       </c>
@@ -45056,7 +45038,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="381" spans="1:34" ht="15" customHeight="1">
+    <row r="381" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A381" s="1" t="s">
         <v>88</v>
       </c>
@@ -45158,7 +45140,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="382" spans="1:34" ht="15" customHeight="1">
+    <row r="382" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A382" s="1" t="s">
         <v>88</v>
       </c>
@@ -45262,7 +45244,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="383" spans="1:34" ht="15" customHeight="1">
+    <row r="383" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A383" s="1" t="s">
         <v>82</v>
       </c>
@@ -45364,7 +45346,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="384" spans="1:34" ht="24" customHeight="1">
+    <row r="384" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A384" s="1" t="s">
         <v>42</v>
       </c>
@@ -45466,7 +45448,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="385" spans="1:34" ht="24" customHeight="1">
+    <row r="385" spans="1:34" ht="24" hidden="1" customHeight="1">
       <c r="A385" s="1" t="s">
         <v>42</v>
       </c>
@@ -45570,7 +45552,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="386" spans="1:34" ht="15" customHeight="1">
+    <row r="386" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A386" s="1" t="s">
         <v>140</v>
       </c>
@@ -45674,7 +45656,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="387" spans="1:34" ht="15" customHeight="1">
+    <row r="387" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A387" s="1" t="s">
         <v>65</v>
       </c>
@@ -45770,7 +45752,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="388" spans="1:34" ht="15" customHeight="1">
+    <row r="388" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A388" s="1" t="s">
         <v>39</v>
       </c>
@@ -45872,7 +45854,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="389" spans="1:34" ht="15" customHeight="1">
+    <row r="389" spans="1:34" ht="15" hidden="1" customHeight="1">
       <c r="A389" s="1" t="s">
         <v>60</v>
       </c>
@@ -66006,7 +65988,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="3" spans="1:18" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>82</v>
       </c>
@@ -66060,7 +66042,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="4" spans="1:18" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>54</v>
       </c>
@@ -66168,7 +66150,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="6" spans="1:18" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>140</v>
       </c>
@@ -66332,7 +66314,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="9" spans="1:18" ht="15" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>82</v>
       </c>
@@ -66440,7 +66422,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="11" spans="1:18" ht="15" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>54</v>
       </c>
@@ -66496,7 +66478,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="12" spans="1:18" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>82</v>
       </c>
@@ -66718,7 +66700,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="16" spans="1:18" ht="15" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>82</v>
       </c>
@@ -66886,7 +66868,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="19" spans="1:18" ht="15" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>140</v>
       </c>
@@ -67050,7 +67032,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="22" spans="1:18" ht="15" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>82</v>
       </c>
@@ -67158,7 +67140,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="24" spans="1:18" ht="15" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
@@ -67266,7 +67248,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="26" spans="1:18" ht="15" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>54</v>
       </c>
@@ -67590,7 +67572,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="32" spans="1:18" ht="15" customHeight="1">
       <c r="A32" s="1" t="s">
         <v>140</v>
       </c>
@@ -67916,7 +67898,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="38" spans="1:18" ht="15" customHeight="1">
       <c r="A38" s="1" t="s">
         <v>91</v>
       </c>
@@ -67972,7 +67954,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="39" spans="1:18" ht="15" customHeight="1">
       <c r="A39" s="1" t="s">
         <v>91</v>
       </c>
@@ -68246,7 +68228,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="44" spans="1:18" ht="15" customHeight="1">
       <c r="A44" s="1" t="s">
         <v>54</v>
       </c>
@@ -68792,7 +68774,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="54" spans="1:18" ht="15" customHeight="1">
       <c r="A54" s="1" t="s">
         <v>101</v>
       </c>
@@ -68902,7 +68884,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="56" spans="1:18" ht="15" customHeight="1">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -69714,7 +69696,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="71" spans="1:18" ht="15" customHeight="1">
       <c r="A71" s="1" t="s">
         <v>101</v>
       </c>
@@ -72056,7 +72038,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="114" spans="1:18" ht="15" customHeight="1">
       <c r="A114" s="1" t="s">
         <v>39</v>
       </c>
@@ -73412,7 +73394,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="139" spans="1:18" ht="15" customHeight="1">
       <c r="A139" s="1" t="s">
         <v>54</v>
       </c>
@@ -78306,7 +78288,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="229" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="229" spans="1:18" ht="15" customHeight="1">
       <c r="A229" s="1" t="s">
         <v>65</v>
       </c>

</xml_diff>

<commit_message>
Atualiza roadmap SEO e AEO
Detalha o monitoramento de AEO por prompts e ajusta as prioridades e KPIs das fases de 0–30, 31–60 e 61–90 dias.
</commit_message>
<xml_diff>
--- a/analise/analise-seo-infinitepay.xlsx
+++ b/analise/analise-seo-infinitepay.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesll\Downloads\Teste Cloudwalk\analise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E7E698-8AE1-460F-B048-265CE438D14E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70F793E-7193-472C-AE2B-3DD32FD0DC5D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arquitetura de páginas" sheetId="11" r:id="rId1"/>
@@ -4233,23 +4233,14 @@
 LANÇAR E CONECTAR</t>
   </si>
   <si>
-    <t>Presença da InfinitePay · URL citada · fontes concorrentes</t>
-  </si>
-  <si>
     <t>31–60 dias
 APRENDER E AMPLIAR</t>
   </si>
   <si>
-    <t>Mudança de presença/citação · fontes que seguem dominando respostas</t>
-  </si>
-  <si>
     <t>61–90 dias
 ESCALAR O QUE FUNCIONOU</t>
   </si>
   <si>
-    <t>Presença/citações vs. baseline · URLs citadas</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -4364,9 +4355,6 @@
     <t>Verificar se o Google encontra a página e registrar a presença inicial nas respostas de IA.</t>
   </si>
   <si>
-    <t>Aproveitar os conteúdos existentes para apoiar o lançamento.</t>
-  </si>
-  <si>
     <t>Analisar no Search Console as buscas que levam à calculadora.</t>
   </si>
   <si>
@@ -4379,9 +4367,6 @@
     <t>Revisar links e presença nas IAs. Criar conteúdo apenas para necessidades diferentes.</t>
   </si>
   <si>
-    <t>Usar os dados reais para orientar os próximos ajustes.</t>
-  </si>
-  <si>
     <t>Melhorar conteúdo e apresentação no Google nas buscas com potencial de ganho.</t>
   </si>
   <si>
@@ -4409,10 +4394,25 @@
     <t>Indexação · impressões · posição · cliques · CTR</t>
   </si>
   <si>
-    <t>Queries · impressões · posição · cliques · CTR</t>
-  </si>
-  <si>
-    <t>Queries · impressões · posição · cliques · CTR · referring domains</t>
+    <t>Garantir a indexação e cadastrar prompts relacionados à ferramenta para criar um baseline de presença nas respostas de IA.</t>
+  </si>
+  <si>
+    <t>Presença da InfinitePay · URL citada · fontes concorrentes (Profound, First Answer, Semrush)</t>
+  </si>
+  <si>
+    <t>Queries · impressões · posição · cliques · CTR · referring domains (GSC e GA4 para MQLs)</t>
+  </si>
+  <si>
+    <t>Queries · impressões · posição · cliques · CT R · referring domains (GSC e GA4 para MQLs)</t>
+  </si>
+  <si>
+    <t>Mudança de presença/citação · fontes que seguem dominando respostas (Profound, First Answer, Semrush)</t>
+  </si>
+  <si>
+    <t>Presença/citações vs. baseline · URLs citadas (Profound, First Answer, Semrush)</t>
+  </si>
+  <si>
+    <t>Monitorar os prompts cadastrados e identificar perguntas, páginas citadas e concorrentes mais presentes nas respostas de IA.</t>
   </si>
 </sst>
 </file>
@@ -5427,6 +5427,11 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Base1" displayName="Base1" ref="A1:AH389" totalsRowShown="0">
   <autoFilter ref="A1:AH389" xr:uid="{DDA5E582-3654-4FFC-8F29-F80B4F9FF6CC}">
+    <filterColumn colId="26">
+      <filters>
+        <filter val="Sim"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="32">
       <filters>
         <filter val="Oportunidade"/>
@@ -5753,140 +5758,140 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="26" t="s">
-        <v>1390</v>
+        <v>1387</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>1441</v>
+        <v>1436</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>1391</v>
+        <v>1388</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>1440</v>
+        <v>1435</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>1392</v>
+        <v>1389</v>
       </c>
       <c r="F1" s="26" t="s">
         <v>1374</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>1393</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="64.95" customHeight="1">
       <c r="A2" s="28" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>1392</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>1393</v>
+      </c>
+      <c r="D2" s="28" t="s">
         <v>1394</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="E2" s="28" t="s">
         <v>1395</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="F2" s="28" t="s">
         <v>1396</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="G2" s="28" t="s">
         <v>1397</v>
-      </c>
-      <c r="E2" s="28" t="s">
-        <v>1398</v>
-      </c>
-      <c r="F2" s="28" t="s">
-        <v>1399</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>1400</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="64.95" customHeight="1">
       <c r="A3" s="25" t="s">
-        <v>1394</v>
+        <v>1391</v>
       </c>
       <c r="B3" s="25" t="s">
+        <v>1398</v>
+      </c>
+      <c r="C3" s="38" t="s">
+        <v>1399</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>1400</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>1401</v>
       </c>
-      <c r="C3" s="38" t="s">
+      <c r="F3" s="25" t="s">
         <v>1402</v>
       </c>
-      <c r="D3" s="25" t="s">
-        <v>1403</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>1404</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>1405</v>
-      </c>
       <c r="G3" s="25" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="64.95" customHeight="1">
       <c r="A4" s="28" t="s">
-        <v>1394</v>
+        <v>1391</v>
       </c>
       <c r="B4" s="28" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C4" s="39" t="s">
+        <v>1404</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>1405</v>
+      </c>
+      <c r="E4" s="28" t="s">
         <v>1406</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="F4" s="28" t="s">
         <v>1407</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="G4" s="28" t="s">
         <v>1408</v>
-      </c>
-      <c r="E4" s="28" t="s">
-        <v>1409</v>
-      </c>
-      <c r="F4" s="28" t="s">
-        <v>1410</v>
-      </c>
-      <c r="G4" s="28" t="s">
-        <v>1411</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="64.95" customHeight="1">
       <c r="A5" s="25" t="s">
-        <v>1412</v>
+        <v>1409</v>
       </c>
       <c r="B5" s="25" t="s">
         <v>1344</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>1439</v>
+        <v>1434</v>
       </c>
       <c r="D5" s="25" t="s">
+        <v>1410</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>1411</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>1412</v>
+      </c>
+      <c r="G5" s="25" t="s">
         <v>1413</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>1414</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>1415</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>1416</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="64.95" customHeight="1">
       <c r="A6" s="28" t="s">
-        <v>1394</v>
+        <v>1391</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>1417</v>
+        <v>1414</v>
       </c>
       <c r="C6" s="39" t="s">
         <v>1314</v>
       </c>
       <c r="D6" s="28" t="s">
+        <v>1415</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>1417</v>
+      </c>
+      <c r="G6" s="28" t="s">
         <v>1418</v>
-      </c>
-      <c r="E6" s="28" t="s">
-        <v>1419</v>
-      </c>
-      <c r="F6" s="28" t="s">
-        <v>1420</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>1421</v>
       </c>
     </row>
   </sheetData>
@@ -5915,7 +5920,7 @@
     <col min="3" max="3" width="42.296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.8984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.19921875" customWidth="1"/>
     <col min="7" max="7" width="19.09765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5" customWidth="1"/>
   </cols>
@@ -5940,10 +5945,10 @@
         <v>1383</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>1422</v>
+        <v>1419</v>
       </c>
       <c r="H1" s="26" t="s">
-        <v>1423</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="79.2">
@@ -5951,77 +5956,77 @@
         <v>1384</v>
       </c>
       <c r="B2" s="33" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>1423</v>
+      </c>
+      <c r="E2" s="34" t="s">
         <v>1424</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="F2" s="17" t="s">
+        <v>1438</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>1437</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="92.4">
+      <c r="A3" s="29" t="s">
+        <v>1385</v>
+      </c>
+      <c r="B3" s="35" t="s">
         <v>1425</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="C3" s="36" t="s">
         <v>1426</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="D3" s="36" t="s">
         <v>1427</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="E3" s="36" t="s">
         <v>1428</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="F3" s="16" t="s">
+        <v>1444</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>1440</v>
+      </c>
+      <c r="H3" s="16" t="s">
         <v>1442</v>
       </c>
-      <c r="H2" s="17" t="s">
-        <v>1385</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="66">
-      <c r="A3" s="29" t="s">
+    </row>
+    <row r="4" spans="1:8" ht="66">
+      <c r="A4" s="37" t="s">
         <v>1386</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B4" s="33" t="s">
         <v>1429</v>
       </c>
-      <c r="C3" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>1430</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D4" s="34" t="s">
         <v>1431</v>
       </c>
-      <c r="E3" s="36" t="s">
+      <c r="E4" s="34" t="s">
         <v>1432</v>
       </c>
-      <c r="F3" s="36" t="s">
+      <c r="F4" s="34" t="s">
         <v>1433</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G4" s="15" t="s">
+        <v>1441</v>
+      </c>
+      <c r="H4" s="15" t="s">
         <v>1443</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>1387</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="52.8">
-      <c r="A4" s="37" t="s">
-        <v>1388</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>1434</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>1435</v>
-      </c>
-      <c r="D4" s="34" t="s">
-        <v>1436</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>1437</v>
-      </c>
-      <c r="F4" s="34" t="s">
-        <v>1438</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>1444</v>
-      </c>
-      <c r="H4" s="15" t="s">
-        <v>1389</v>
       </c>
     </row>
     <row r="5" spans="1:8">

</xml_diff>